<commit_message>
updated BOM and schematics
</commit_message>
<xml_diff>
--- a/Aegis Grid/resources/BOM/BOM.xlsx
+++ b/Aegis Grid/resources/BOM/BOM.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicoj\iCloudDrive\McMaster Important Stuff\Year 4\Semester 1\IoT Devices and Networks - SMRTTECH 4ID3\GROUP PROJECT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicoj\Documents\Repositories\4ID3\Aegis Grid\resources\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96048205-DDC4-4EC9-84A9-EF2AC2873793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C0AA80-E751-4746-82DE-808F457C5337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{196CD192-2C0A-48B9-ABAB-C59F140B49E5}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{196CD192-2C0A-48B9-ABAB-C59F140B49E5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="other tables" sheetId="2" r:id="rId2"/>
+    <sheet name="BOM Proof-of-Concept" sheetId="1" r:id="rId1"/>
+    <sheet name="BOM Industrial Comparison" sheetId="3" r:id="rId2"/>
+    <sheet name="other tables" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="70">
   <si>
     <t>Qty</t>
   </si>
@@ -54,9 +55,6 @@
     <t>Red LED</t>
   </si>
   <si>
-    <t>we have</t>
-  </si>
-  <si>
     <t>breadboard</t>
   </si>
   <si>
@@ -117,25 +115,139 @@
     <t>MacIoT board</t>
   </si>
   <si>
-    <t>active or passive buzzer</t>
-  </si>
-  <si>
     <t>DC motor</t>
   </si>
   <si>
-    <t>DHT11 humidity sensor</t>
-  </si>
-  <si>
-    <t>TMP36 temperature sensor</t>
-  </si>
-  <si>
-    <t>Low offset voltage dual comparators</t>
-  </si>
-  <si>
     <t>Piezoelectric ceramic vibration sensor module</t>
   </si>
   <si>
-    <t>Shunt resistor</t>
+    <t>On Hand</t>
+  </si>
+  <si>
+    <t>passive buzzer</t>
+  </si>
+  <si>
+    <t>EBYTE LoRa module</t>
+  </si>
+  <si>
+    <t>1k resistor</t>
+  </si>
+  <si>
+    <t>a bunch</t>
+  </si>
+  <si>
+    <t>wires</t>
+  </si>
+  <si>
+    <t>9V battery</t>
+  </si>
+  <si>
+    <t>potentiometer</t>
+  </si>
+  <si>
+    <t>220 resistor</t>
+  </si>
+  <si>
+    <t>DHT11 temperature &amp; humidity sensor</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Proof-of-Concept Component</t>
+  </si>
+  <si>
+    <t>Industrial Solution Component</t>
+  </si>
+  <si>
+    <t>Field Device</t>
+  </si>
+  <si>
+    <t>Gateway Device</t>
+  </si>
+  <si>
+    <t>LoRa Module</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Planet LCG-300</t>
+  </si>
+  <si>
+    <t>Vibration Sensor</t>
+  </si>
+  <si>
+    <t>Daviteq WSLRW-V1A</t>
+  </si>
+  <si>
+    <t>Milesight EM500-PT100</t>
+  </si>
+  <si>
+    <t>Red LEDs Passive Buzzers</t>
+  </si>
+  <si>
+    <t>Alarm</t>
+  </si>
+  <si>
+    <t>Patlite LR5 Signal Tower</t>
+  </si>
+  <si>
+    <t>Application Software</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>IBM Maximo Health and Predict Utilities</t>
+  </si>
+  <si>
+    <t>IoT Network Management</t>
+  </si>
+  <si>
+    <t>Node-RED</t>
+  </si>
+  <si>
+    <t>AWS IoT Core for LoRaWAN</t>
+  </si>
+  <si>
+    <t>Voltage/Current Sensors</t>
+  </si>
+  <si>
+    <t>MacIoT board Analog Pins</t>
+  </si>
+  <si>
+    <t>CT/PT Transformer Step-Down to Meters</t>
+  </si>
+  <si>
+    <t>Network Transport</t>
+  </si>
+  <si>
+    <t>MQTT over Wi-Fi</t>
+  </si>
+  <si>
+    <t>MQTT over Ethernet</t>
+  </si>
+  <si>
+    <t>Network Access Protocol</t>
+  </si>
+  <si>
+    <t>LoRa</t>
+  </si>
+  <si>
+    <t>LoRaWAN</t>
+  </si>
+  <si>
+    <t>Power Grid Equipment</t>
+  </si>
+  <si>
+    <t>DC Motor</t>
+  </si>
+  <si>
+    <t>Generators, Transformers, Transmission Lines, etc.</t>
+  </si>
+  <si>
+    <t>Temperature/Humidity Sensor</t>
   </si>
 </sst>
 </file>
@@ -178,7 +290,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -187,13 +299,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -211,12 +329,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -233,15 +347,25 @@
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -577,253 +701,486 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA0F12EA-53DA-4D28-AF32-40BEC296018C}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="38.7265625" customWidth="1"/>
-    <col min="3" max="3" width="17.90625" customWidth="1"/>
-    <col min="4" max="4" width="9.08984375" style="6"/>
+    <col min="1" max="1" width="9.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="38.90625" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="5">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="3">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="1">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="1">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="7">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="3">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="7">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="3">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="1">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="7">
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C15" s="13" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="3">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="3">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" s="7">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="3">
-        <v>2</v>
-      </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="7">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="3">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="3">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="8">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="3">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="8">
+      <c r="D15" s="6">
         <f>SUM(D2:D11)</f>
-        <v>80</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{33A6F2E6-90E8-470F-9C05-6200061A8722}"/>
-    <hyperlink ref="C5" r:id="rId2" xr:uid="{26A2833F-2D19-4DB7-9232-720DA22BAF72}"/>
-    <hyperlink ref="C6" r:id="rId3" xr:uid="{A3E1F4B9-F4D3-4E84-A433-C8BBB65DBA00}"/>
-    <hyperlink ref="C7" r:id="rId4" xr:uid="{5F31F05A-F4CB-4AEB-8417-3A45EE128377}"/>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{26A2833F-2D19-4DB7-9232-720DA22BAF72}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ECDC68B-46D5-43B2-A9A2-38B6B056D0B1}">
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="28.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="38.90625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="40.81640625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B15"/>
+      <c r="C15"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B16"/>
+      <c r="C16"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17"/>
+      <c r="C17"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18"/>
+      <c r="C18"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19"/>
+      <c r="C19"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20"/>
+      <c r="C20"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{742CB20E-E5DD-4260-904B-55E33C9B709B}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.7265625" customWidth="1"/>
-    <col min="2" max="2" width="31.453125" style="11" customWidth="1"/>
-    <col min="3" max="3" width="32.81640625" style="11" customWidth="1"/>
+    <col min="1" max="1" width="28.36328125" customWidth="1"/>
+    <col min="2" max="2" width="38.90625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="61.26953125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="9.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>13</v>
+      <c r="C1" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>18</v>
+      <c r="C2" s="9" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="C3" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>22</v>
+      <c r="C4" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>23</v>
+      <c r="C5" s="9" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
initial commit of slideshow for investors
</commit_message>
<xml_diff>
--- a/Aegis Grid/resources/BOM/BOM.xlsx
+++ b/Aegis Grid/resources/BOM/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicoj\Documents\Repositories\4ID3\Aegis Grid\resources\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C0AA80-E751-4746-82DE-808F457C5337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC4E518E-5AD0-44F1-8260-4622C4B9800B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{196CD192-2C0A-48B9-ABAB-C59F140B49E5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{196CD192-2C0A-48B9-ABAB-C59F140B49E5}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM Proof-of-Concept" sheetId="1" r:id="rId1"/>
@@ -311,7 +311,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.499984740745262"/>
+        <fgColor theme="1" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -931,7 +931,7 @@
   <cols>
     <col min="1" max="1" width="28.1796875" style="1" customWidth="1"/>
     <col min="2" max="2" width="38.90625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="40.81640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="42.6328125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>